<commit_message>
Version 03 efa vita migration - efa configure ny admin zany hoe ny authentification zany efa ok
</commit_message>
<xml_diff>
--- a/etape.xlsx
+++ b/etape.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Projet en General</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t xml:space="preserve"> 🆗 Etapes </t>
+  </si>
+  <si>
+    <t>python manage.py creatsuperuser</t>
   </si>
 </sst>
 </file>
@@ -127,8 +130,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -136,8 +139,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -440,11 +443,11 @@
       <c r="I1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -456,82 +459,82 @@
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
       <c r="J4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
       <c r="J6" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
@@ -544,9 +547,9 @@
       <c r="I9" s="5"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -555,14 +558,16 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="B11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>

</xml_diff>